<commit_message>
exp results strategy eval
</commit_message>
<xml_diff>
--- a/results/reliability_eval/unified_scores_table_08-24-3.xlsx
+++ b/results/reliability_eval/unified_scores_table_08-24-3.xlsx
@@ -431,188 +431,188 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Dataset Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Beam Search</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Max New Tokens</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>AUCROC_sample</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_sample</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AUCROC_adj</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_adj</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>AUCROC_entr</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_entr</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>AUCROC_sem</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_sem</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Dataset Name</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Beam Search</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Max New Tokens</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Strategy</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.4190981432360743</v>
       </c>
-      <c r="B2" t="n">
+      <c r="I2" t="n">
         <v>0.1308952862555237</v>
       </c>
-      <c r="C2" t="n">
+      <c r="J2" t="n">
         <v>0.4190981432360743</v>
       </c>
-      <c r="D2" t="n">
+      <c r="K2" t="n">
         <v>0.1308952862555237</v>
       </c>
-      <c r="E2" t="n">
+      <c r="L2" t="n">
         <v>0.4801061007957561</v>
       </c>
-      <c r="F2" t="n">
+      <c r="M2" t="n">
         <v>0.1261792580932974</v>
       </c>
-      <c r="G2" t="n">
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="n">
+      <c r="O2" t="n">
         <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Llama-3-8B</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>P101</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>beam</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>10</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>fact_statement</t>
-        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.975</v>
       </c>
-      <c r="B3" t="n">
+      <c r="I3" t="n">
         <v>0.9930555555555556</v>
       </c>
-      <c r="C3" t="n">
+      <c r="J3" t="n">
         <v>0.975</v>
       </c>
-      <c r="D3" t="n">
+      <c r="K3" t="n">
         <v>0.9930555555555556</v>
       </c>
-      <c r="E3" t="n">
+      <c r="L3" t="n">
         <v>0.225</v>
       </c>
-      <c r="F3" t="n">
+      <c r="M3" t="n">
         <v>0.6500599549336971</v>
       </c>
-      <c r="G3" t="n">
+      <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" t="n">
+      <c r="O3" t="n">
         <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.7619047619047619</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Llama-3-8B</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>toy-qa-dataset</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>beam</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>10</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>fact_statement</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>